<commit_message>
fix: enforce business-complete document workflows
</commit_message>
<xml_diff>
--- a/tests/manual/03-表格填充/05-极限-经营驾驶舱/期望结果.xlsx
+++ b/tests/manual/03-表格填充/05-极限-经营驾驶舱/期望结果.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="区域经营" sheetId="1" r:id="R1571907e53a84c57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度明细" sheetId="2" r:id="Rdebcdc563e664523"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="异常说明" sheetId="3" r:id="R6437c4b3942d4e9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="区域经营" sheetId="1" r:id="Rde2b074d193c4a6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月度明细" sheetId="2" r:id="Rf32c4031600d4e46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="异常说明" sheetId="3" r:id="R4a73656816444d3f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -341,25 +341,25 @@
         <x:v>华东</x:v>
       </x:c>
       <x:c r="B2" s="8" t="n">
-        <x:v>1312</x:v>
+        <x:v>1372</x:v>
       </x:c>
       <x:c r="C2" s="8" t="n">
         <x:v>865</x:v>
       </x:c>
       <x:c r="D2" s="8" t="n">
         <x:f>B2-C2</x:f>
-        <x:v>447</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="E2" s="9" t="n">
         <x:f>D2/B2</x:f>
-        <x:v>0.3407012195121951</x:v>
+        <x:v>0.369533527696793</x:v>
       </x:c>
       <x:c r="F2" s="8" t="n">
         <x:v>1450</x:v>
       </x:c>
       <x:c r="G2" s="9" t="n">
         <x:f>B2/F2</x:f>
-        <x:v>0.9048275862068965</x:v>
+        <x:v>0.9462068965517242</x:v>
       </x:c>
     </x:row>
     <x:row r="3">

</xml_diff>